<commit_message>
agentes y data junio 3
</commit_message>
<xml_diff>
--- a/data/raw/Ficha_Tecnica_Indicadores.xlsx
+++ b/data/raw/Ficha_Tecnica_Indicadores.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5f15395a9ed9a48f/Proyectos_DS/Sistema_Indicadores_Poli/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="51" documentId="8_{14DDC1C0-2002-47F7-B3C5-8322D3D19E2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{13E6041E-E5ED-4E5F-BE91-9033715DD1D3}"/>
+  <xr:revisionPtr revIDLastSave="52" documentId="8_{14DDC1C0-2002-47F7-B3C5-8322D3D19E2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{98A3573A-E951-4894-ACE6-0F0DAE171675}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DC62A0ED-0F95-4A2B-9410-ED2E5065736A}"/>
+    <workbookView xWindow="5604" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{DC62A0ED-0F95-4A2B-9410-ED2E5065736A}"/>
   </bookViews>
   <sheets>
     <sheet name="query (1)" sheetId="1" r:id="rId1"/>
@@ -11924,7 +11924,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -12686,7 +12686,9 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{6FB43CA5-EC4C-482A-A6AB-275F607DEA8C}"/>
+  </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>

</xml_diff>